<commit_message>
docs: update project spreadsheets
</commit_message>
<xml_diff>
--- a/doc/行知旅伴_V2.3_产品待办列表_含负责人.xlsx
+++ b/doc/行知旅伴_V2.3_产品待办列表_含负责人.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版权说明" sheetId="1" r:id="R642a708d85394bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品Backlog" sheetId="2" r:id="R9dc3a79dfce64075"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="团队速率" sheetId="3" r:id="R5ab0135f2c034990"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版权说明" sheetId="1" r:id="R25a4059023d847a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品Backlog" sheetId="2" r:id="R0f82a6db078e476a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="团队速率" sheetId="3" r:id="Ra92acd7c38984397"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="201" formatCode="0.0"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -83,8 +83,14 @@
       <x:color rgb="FF111827"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -144,6 +150,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -309,7 +320,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="141">
+  <x:cellXfs count="144">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -634,6 +645,11 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -700,7 +716,7 @@
         <x:color rgb="FF7C4A03"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -1282,7 +1298,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M7" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="126" customHeight="1">
@@ -1328,7 +1344,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M8" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="126" customHeight="1">
@@ -1374,7 +1390,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M9" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="126" customHeight="1">
@@ -1420,7 +1436,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M10" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="126" customHeight="1">
@@ -1466,7 +1482,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M11" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="126" customHeight="1">
@@ -1512,7 +1528,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M12" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="126" customHeight="1">
@@ -1558,7 +1574,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M13" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="126" customHeight="1">
@@ -1604,7 +1620,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M14" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="126" customHeight="1">
@@ -1650,7 +1666,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M15" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="126" customHeight="1">
@@ -1696,7 +1712,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M16" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="126" customHeight="1">
@@ -1742,7 +1758,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="M17" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="126" customHeight="1">
@@ -1788,7 +1804,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M18" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="126" customHeight="1">
@@ -1834,7 +1850,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M19" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>基本完成，待最终验收</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="126" customHeight="1">
@@ -1880,7 +1896,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M20" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>基本完成，待最终验收</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="126" customHeight="1">
@@ -1926,7 +1942,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M21" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>基本完成，待最终验收</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="126" customHeight="1">
@@ -1972,7 +1988,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M22" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>基本完成，待最终验收</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="126" customHeight="1">
@@ -2018,7 +2034,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M23" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>基本完成，待最终验收</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="126" customHeight="1">
@@ -2064,7 +2080,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M24" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>基本完成，待最终验收</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="126" customHeight="1">
@@ -2110,7 +2126,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M25" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>基本完成，待最终验收</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="126" customHeight="1">
@@ -2156,7 +2172,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M26" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>基本完成，待最终验收</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="126" customHeight="1">
@@ -2202,7 +2218,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M27" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>待执行</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="126" customHeight="1">
@@ -2248,7 +2264,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M28" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>待执行</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="126" customHeight="1">
@@ -2294,7 +2310,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="M29" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>待执行</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="126" customHeight="1">
@@ -2340,7 +2356,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M30" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>待执行</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="126" customHeight="1">
@@ -2386,7 +2402,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M31" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>待执行</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="126" customHeight="1">
@@ -2432,7 +2448,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M32" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>待执行</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="126" customHeight="1">
@@ -2478,7 +2494,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="M33" s="94" t="str">
-        <x:v>待办</x:v>
+        <x:v>待执行</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="126" customHeight="1">
@@ -2618,6 +2634,25 @@
       <x:c r="M36" s="94" t="str">
         <x:v>候选池</x:v>
       </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="143" t="str">
+        <x:v>调整说明</x:v>
+      </x:c>
+      <x:c r="B38" s="143" t="str">
+        <x:v>Sprint1 已完成；Sprint2 开发主链基本完成，仅保留公网/设备最终验收；Sprint3 纳入原始 PBI-13-S3 至 PBI-17 以及 Sprint2 最终验收收尾。</x:v>
+      </x:c>
+      <x:c r="C38" s="143"/>
+      <x:c r="D38" s="143"/>
+      <x:c r="E38" s="143"/>
+      <x:c r="F38" s="143"/>
+      <x:c r="G38" s="143"/>
+      <x:c r="H38" s="143"/>
+      <x:c r="I38" s="143"/>
+      <x:c r="J38" s="143"/>
+      <x:c r="K38" s="143"/>
+      <x:c r="L38" s="143"/>
+      <x:c r="M38" s="143"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>